<commit_message>
After reafactor, handoffs, tax earned report
</commit_message>
<xml_diff>
--- a/Austerlitz/Turns/Online Austerlitz - Spain 436.xlsx
+++ b/Austerlitz/Turns/Online Austerlitz - Spain 436.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Austerlitz\436\Mar 1808\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB3F12BF-D28D-466C-9C71-47AFEA6CD258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC821547-FD6B-4383-B660-EBEDC028650F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="76">
   <si>
     <t>A U S T E R L I T Z</t>
   </si>
@@ -252,6 +252,18 @@
   </si>
   <si>
     <t>(23) Change State Relationships  (State/New Relationship)</t>
+  </si>
+  <si>
+    <t>5th Rifles</t>
+  </si>
+  <si>
+    <t>6th Rifles</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>03.08.26</t>
   </si>
 </sst>
 </file>
@@ -884,8 +896,8 @@
         <v>9</v>
       </c>
       <c r="F7" s="6"/>
-      <c r="G7" s="28">
-        <v>46237</v>
+      <c r="G7" s="28" t="s">
+        <v>75</v>
       </c>
       <c r="H7" s="28"/>
       <c r="I7" s="28"/>
@@ -1111,18 +1123,28 @@
       <c r="A16" s="6">
         <v>5</v>
       </c>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
+      <c r="B16" s="13">
+        <v>1</v>
+      </c>
+      <c r="C16" s="13">
+        <v>203</v>
+      </c>
+      <c r="D16" s="13">
+        <v>1040000</v>
+      </c>
+      <c r="E16" s="13">
+        <v>8000</v>
+      </c>
+      <c r="F16" s="13">
+        <v>1600</v>
+      </c>
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>Valid</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="13.5" customHeight="1">
@@ -1467,15 +1489,29 @@
       <c r="A34" s="6">
         <v>1</v>
       </c>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
+      <c r="B34" s="11">
+        <v>203</v>
+      </c>
+      <c r="C34" s="11">
+        <v>11</v>
+      </c>
+      <c r="D34" s="11">
+        <v>11</v>
+      </c>
+      <c r="E34" s="11">
+        <v>11</v>
+      </c>
+      <c r="F34" s="11">
+        <v>11</v>
+      </c>
+      <c r="G34" s="11">
+        <v>11</v>
+      </c>
       <c r="H34" s="11"/>
       <c r="I34" s="13"/>
-      <c r="J34" s="11"/>
+      <c r="J34" s="11" t="s">
+        <v>72</v>
+      </c>
       <c r="K34" s="7"/>
       <c r="L34" s="7" t="str">
         <f t="shared" ref="L34:L41" si="2">IF(AND(B34="",C34="",D34="",E34="",F34="",G34="",H34="",I34="",J34=""),"",
@@ -1495,26 +1531,40 @@
 IF(AND(I34&lt;&gt;"",OR(C34="",D34="",E34="",F34="",G34="",H34="")),"Battalion 7 requires all previous battalions",
 IF(J34="","Name is required",
 IF(LEN(J34)&gt;15,"Name must not exceed 15 characters","Valid")))))))))))</f>
-        <v/>
+        <v>Valid</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="13.5" customHeight="1">
       <c r="A35" s="6">
         <v>2</v>
       </c>
-      <c r="B35" s="13"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
+      <c r="B35" s="13">
+        <v>203</v>
+      </c>
+      <c r="C35" s="11">
+        <v>11</v>
+      </c>
+      <c r="D35" s="11">
+        <v>11</v>
+      </c>
+      <c r="E35" s="11">
+        <v>11</v>
+      </c>
+      <c r="F35" s="11">
+        <v>11</v>
+      </c>
+      <c r="G35" s="11">
+        <v>11</v>
+      </c>
       <c r="H35" s="13"/>
       <c r="I35" s="13"/>
-      <c r="J35" s="11"/>
+      <c r="J35" s="11" t="s">
+        <v>73</v>
+      </c>
       <c r="K35" s="7"/>
       <c r="L35" s="7" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Valid</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="13.5" customHeight="1">
@@ -3578,8 +3628,12 @@
       <c r="A133" s="6">
         <v>1</v>
       </c>
-      <c r="B133" s="13"/>
-      <c r="C133" s="13"/>
+      <c r="B133" s="13">
+        <v>15</v>
+      </c>
+      <c r="C133" s="13">
+        <v>43</v>
+      </c>
       <c r="D133" s="6"/>
       <c r="E133" s="6"/>
       <c r="F133" s="6"/>
@@ -3618,8 +3672,12 @@
       <c r="A134" s="6">
         <v>2</v>
       </c>
-      <c r="B134" s="13"/>
-      <c r="C134" s="13"/>
+      <c r="B134" s="13">
+        <v>16</v>
+      </c>
+      <c r="C134" s="13">
+        <v>36</v>
+      </c>
       <c r="D134" s="6"/>
       <c r="E134" s="6"/>
       <c r="F134" s="6"/>
@@ -3658,8 +3716,12 @@
       <c r="A135" s="6">
         <v>3</v>
       </c>
-      <c r="B135" s="13"/>
-      <c r="C135" s="13"/>
+      <c r="B135" s="13">
+        <v>18</v>
+      </c>
+      <c r="C135" s="13">
+        <v>36</v>
+      </c>
       <c r="D135" s="6"/>
       <c r="E135" s="6"/>
       <c r="F135" s="6"/>
@@ -3698,8 +3760,12 @@
       <c r="A136" s="6">
         <v>4</v>
       </c>
-      <c r="B136" s="13"/>
-      <c r="C136" s="11"/>
+      <c r="B136" s="13">
+        <v>19</v>
+      </c>
+      <c r="C136" s="11">
+        <v>37</v>
+      </c>
       <c r="D136" s="6"/>
       <c r="E136" s="6"/>
       <c r="F136" s="6"/>
@@ -3738,8 +3804,12 @@
       <c r="A137" s="6">
         <v>5</v>
       </c>
-      <c r="B137" s="13"/>
-      <c r="C137" s="13"/>
+      <c r="B137" s="13">
+        <v>20</v>
+      </c>
+      <c r="C137" s="13">
+        <v>38</v>
+      </c>
       <c r="D137" s="6"/>
       <c r="E137" s="6"/>
       <c r="F137" s="6"/>
@@ -12623,9 +12693,11 @@
         <v>1</v>
       </c>
       <c r="B304" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C304" s="13"/>
+        <v>74</v>
+      </c>
+      <c r="C304" s="13">
+        <v>4</v>
+      </c>
       <c r="D304" s="6"/>
       <c r="E304" s="6"/>
       <c r="F304" s="6"/>

</xml_diff>